<commit_message>
Sync code from nested directory and resolve merge conflicts. Update Dashboard with integrated Recent Tests and AllSamples page.
</commit_message>
<xml_diff>
--- a/lims_backend/lab_data.xlsx
+++ b/lims_backend/lab_data.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13.21875" customWidth="1" min="3" max="3"/>
@@ -527,6 +527,195 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S-2026-2050-ABC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B-1230</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ORD-22005</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Admin01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S-2026-2222</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B-1000</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ORD-15402</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NPK</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.21</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Admin01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>04:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S-2026-2808</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B-1000</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ORD-154</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NPK</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>99.99</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Admin01</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>17:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S-2026-28035</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B-1023</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ORD-154023</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Admolh</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>18:56</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>